<commit_message>
Privacy-harden Excel portfolio demo data
</commit_message>
<xml_diff>
--- a/excel-projects/RA_Customer_Service_SLA_Dashboard.xlsx
+++ b/excel-projects/RA_Customer_Service_SLA_Dashboard.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R57503bd4c8394faf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="2" r:id="Rf989315c08ef497f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agents" sheetId="3" r:id="R25dafbceb89c434c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rc4626b1d84df488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rc176f9ebf1794d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tickets" sheetId="2" r:id="R20869d34099c4c68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agents" sheetId="3" r:id="Rea962ac656644b0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rfb8fb4c4bc0a4898"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -159,7 +159,7 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -169,7 +169,7 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -179,7 +179,7 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -438,7 +438,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R28a6d0b9a943492b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdc6424f13dfa4946"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -468,7 +468,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4f81076e55f445ea"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5a8a3ddcc814c5b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -908,7 +908,7 @@
     <x:row r="19">
       <x:c r="A19" t="str">
         <x:f>Agents!A2</x:f>
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="B19" t="n">
         <x:f>Agents!B2</x:f>
@@ -934,7 +934,7 @@
     <x:row r="20">
       <x:c r="A20" t="str">
         <x:f>Agents!A3</x:f>
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="B20" t="n">
         <x:f>Agents!B3</x:f>
@@ -960,7 +960,7 @@
     <x:row r="21">
       <x:c r="A21" t="str">
         <x:f>Agents!A4</x:f>
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="B21" t="n">
         <x:f>Agents!B4</x:f>
@@ -986,7 +986,7 @@
     <x:row r="22">
       <x:c r="A22" t="str">
         <x:f>Agents!A5</x:f>
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="B22" t="n">
         <x:f>Agents!B5</x:f>
@@ -1012,7 +1012,7 @@
     <x:row r="23">
       <x:c r="A23" t="str">
         <x:f>Agents!A6</x:f>
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="B23" t="n">
         <x:f>Agents!B6</x:f>
@@ -1057,7 +1057,7 @@
     <x:mergeCell ref="G8:H8"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14cbe0a11d984092"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7f7cba7cf024a9a"/>
 </x:worksheet>
 </file>
 
@@ -1129,7 +1129,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>Billing</x:v>
@@ -1164,7 +1164,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D3" t="str">
         <x:v>Technical</x:v>
@@ -1205,7 +1205,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D4" t="str">
         <x:v>Delivery</x:v>
@@ -1246,7 +1246,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Account</x:v>
@@ -1287,7 +1287,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>General</x:v>
@@ -1328,7 +1328,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>Billing</x:v>
@@ -1363,7 +1363,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D8" t="str">
         <x:v>Technical</x:v>
@@ -1404,7 +1404,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D9" t="str">
         <x:v>Delivery</x:v>
@@ -1445,7 +1445,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D10" t="str">
         <x:v>Account</x:v>
@@ -1486,7 +1486,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D11" t="str">
         <x:v>General</x:v>
@@ -1527,7 +1527,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D12" t="str">
         <x:v>Billing</x:v>
@@ -1562,7 +1562,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D13" t="str">
         <x:v>Technical</x:v>
@@ -1603,7 +1603,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D14" t="str">
         <x:v>Delivery</x:v>
@@ -1644,7 +1644,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D15" t="str">
         <x:v>Account</x:v>
@@ -1685,7 +1685,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D16" t="str">
         <x:v>General</x:v>
@@ -1726,7 +1726,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D17" t="str">
         <x:v>Billing</x:v>
@@ -1761,7 +1761,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D18" t="str">
         <x:v>Technical</x:v>
@@ -1802,7 +1802,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D19" t="str">
         <x:v>Delivery</x:v>
@@ -1843,7 +1843,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D20" t="str">
         <x:v>Account</x:v>
@@ -1884,7 +1884,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D21" t="str">
         <x:v>General</x:v>
@@ -1925,7 +1925,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C22" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D22" t="str">
         <x:v>Billing</x:v>
@@ -1960,7 +1960,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C23" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D23" t="str">
         <x:v>Technical</x:v>
@@ -2001,7 +2001,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C24" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D24" t="str">
         <x:v>Delivery</x:v>
@@ -2042,7 +2042,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C25" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D25" t="str">
         <x:v>Account</x:v>
@@ -2083,7 +2083,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D26" t="str">
         <x:v>General</x:v>
@@ -2124,7 +2124,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D27" t="str">
         <x:v>Billing</x:v>
@@ -2159,7 +2159,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D28" t="str">
         <x:v>Technical</x:v>
@@ -2200,7 +2200,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C29" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D29" t="str">
         <x:v>Delivery</x:v>
@@ -2241,7 +2241,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C30" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D30" t="str">
         <x:v>Account</x:v>
@@ -2282,7 +2282,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C31" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D31" t="str">
         <x:v>General</x:v>
@@ -2323,7 +2323,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C32" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D32" t="str">
         <x:v>Billing</x:v>
@@ -2358,7 +2358,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C33" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D33" t="str">
         <x:v>Technical</x:v>
@@ -2399,7 +2399,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C34" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D34" t="str">
         <x:v>Delivery</x:v>
@@ -2440,7 +2440,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C35" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D35" t="str">
         <x:v>Account</x:v>
@@ -2481,7 +2481,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C36" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D36" t="str">
         <x:v>General</x:v>
@@ -2522,7 +2522,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C37" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D37" t="str">
         <x:v>Billing</x:v>
@@ -2557,7 +2557,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C38" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D38" t="str">
         <x:v>Technical</x:v>
@@ -2598,7 +2598,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C39" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D39" t="str">
         <x:v>Delivery</x:v>
@@ -2639,7 +2639,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C40" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D40" t="str">
         <x:v>Account</x:v>
@@ -2680,7 +2680,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D41" t="str">
         <x:v>General</x:v>
@@ -2721,7 +2721,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D42" t="str">
         <x:v>Billing</x:v>
@@ -2756,7 +2756,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C43" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D43" t="str">
         <x:v>Technical</x:v>
@@ -2797,7 +2797,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C44" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D44" t="str">
         <x:v>Delivery</x:v>
@@ -2838,7 +2838,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C45" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D45" t="str">
         <x:v>Account</x:v>
@@ -2879,7 +2879,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C46" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D46" t="str">
         <x:v>General</x:v>
@@ -2920,7 +2920,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C47" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D47" t="str">
         <x:v>Billing</x:v>
@@ -2955,7 +2955,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C48" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D48" t="str">
         <x:v>Technical</x:v>
@@ -2996,7 +2996,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C49" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D49" t="str">
         <x:v>Delivery</x:v>
@@ -3037,7 +3037,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C50" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D50" t="str">
         <x:v>Account</x:v>
@@ -3078,7 +3078,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C51" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D51" t="str">
         <x:v>General</x:v>
@@ -3119,7 +3119,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C52" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D52" t="str">
         <x:v>Billing</x:v>
@@ -3154,7 +3154,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D53" t="str">
         <x:v>Technical</x:v>
@@ -3195,7 +3195,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D54" t="str">
         <x:v>Delivery</x:v>
@@ -3236,7 +3236,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D55" t="str">
         <x:v>Account</x:v>
@@ -3277,7 +3277,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D56" t="str">
         <x:v>General</x:v>
@@ -3318,7 +3318,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="D57" t="str">
         <x:v>Billing</x:v>
@@ -3353,7 +3353,7 @@
         <x:v>Email</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="D58" t="str">
         <x:v>Technical</x:v>
@@ -3394,7 +3394,7 @@
         <x:v>Phone</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="D59" t="str">
         <x:v>Delivery</x:v>
@@ -3435,7 +3435,7 @@
         <x:v>Chat</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="D60" t="str">
         <x:v>Account</x:v>
@@ -3476,7 +3476,7 @@
         <x:v>Web</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="D61" t="str">
         <x:v>General</x:v>
@@ -3539,7 +3539,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0e3cd86e52f4ef4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R360e570448a64475"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3578,7 +3578,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>A. Hassan</x:v>
+        <x:v>Agent A</x:v>
       </x:c>
       <x:c r="B2" t="n">
         <x:f>COUNTIF(Tickets!$C$2:$C$61,A2)</x:f>
@@ -3603,7 +3603,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>M. Khan</x:v>
+        <x:v>Agent B</x:v>
       </x:c>
       <x:c r="B3" t="n">
         <x:f>COUNTIF(Tickets!$C$2:$C$61,A3)</x:f>
@@ -3628,7 +3628,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>S. Omar</x:v>
+        <x:v>Agent C</x:v>
       </x:c>
       <x:c r="B4" t="n">
         <x:f>COUNTIF(Tickets!$C$2:$C$61,A4)</x:f>
@@ -3653,7 +3653,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>N. Ali</x:v>
+        <x:v>Agent D</x:v>
       </x:c>
       <x:c r="B5" t="n">
         <x:f>COUNTIF(Tickets!$C$2:$C$61,A5)</x:f>
@@ -3678,7 +3678,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>F. Saleh</x:v>
+        <x:v>Agent E</x:v>
       </x:c>
       <x:c r="B6" t="n">
         <x:f>COUNTIF(Tickets!$C$2:$C$61,A6)</x:f>

</xml_diff>